<commit_message>
docs: replace P31 with complete accepted manuscript from UWE repository
기존 P31 Holt et al. (2019) 원고본은 표지와 Table 1–4가 빠져 있었습니다.
UWE 기관 저장소의 최종 저자 원고본(26쪽, 표지·Table 1–4 포함)으로
교체합니다. 파일명은 그대로입니다.

- 마스터 P31 행 확인 상태: 표지·Table 1–4 없음 → UWE 저장소, 표지·Table 1–4 포함
- README의 P31 설명 갱신

Refs #13

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
+++ b/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
@@ -4055,7 +4055,7 @@
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23 / 저자 원고본 확인(표지·Table 1–4 없음)</t>
+          <t>2026-10-23 / 저자 원고본 확인(UWE 저장소, 표지·Table 1–4 포함)</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="K127" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23 / 저자 원고본 확인(표지·Table 1–4 없음)</t>
+          <t>2026-10-23 / 저자 원고본 확인(UWE 저장소, 표지·Table 1–4 포함)</t>
         </is>
       </c>
     </row>
@@ -10753,7 +10753,7 @@
       </c>
       <c r="K191" s="6" t="inlineStr">
         <is>
-          <t>2026-10-23 / 저자 원고본 확인(표지·Table 1–4 없음)</t>
+          <t>2026-10-23 / 저자 원고본 확인(UWE 저장소, 표지·Table 1–4 포함)</t>
         </is>
       </c>
     </row>
@@ -13695,7 +13695,7 @@
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23 / 저자 원고본 확인(표지·Table 1–4 없음)</t>
+          <t>2026-10-23 / 저자 원고본 확인(UWE 저장소, 표지·Table 1–4 포함)</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: replace N15 accepted manuscript with ScienceDirect published version
N15 Ratcliffe et al. (2013)의 Surrey 저장소 저자 원고본(표지 포함 31쪽)을
기관 구독(인천대학교) ScienceDirect 출판본(8쪽, 텍스트 PDF)으로 교체합니다.
파일명은 그대로입니다.

- 마스터 N15 행 확인 상태 → 원문 PDF 확인
- R5 결과요약을 원문 기준으로 보강(성인 20명 면담, 새소리별 차이)

Refs #15

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
+++ b/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
@@ -5921,7 +5921,7 @@
       </c>
       <c r="K103" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -9528,7 +9528,7 @@
       </c>
       <c r="H169" s="5" t="inlineStr">
         <is>
-          <t>측정 지표: 지각된 회복성; 새소리 연관; 결과요약: 새소리 종류와 개인 연상에 따라 지각이 달라짐</t>
+          <t>측정 지표: 지각된 회복성; 새소리 연관; 결과요약: 성인 20명 면담에서 새소리가 스트레스 회복·주의 회복과 가장 많이 연관된 자연 소리였으나 모든 새소리가 도움이 되지는 않았고, 지각은 새소리 종류와 개인 연상에 따라 달라짐</t>
         </is>
       </c>
       <c r="I169" s="5" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="K169" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -12435,7 +12435,7 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>초록 확인</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: add six previously missing papers (E20, N11, N13, N19, N22, N25)
미확보였던 마스터 목록 논문 6편의 출판본 텍스트 PDF를 추가합니다.

- 기관 구독(인천대학교) ScienceDirect 5편: E20 Scott et al. (2026),
  N11 Laumann et al. (2001), N13 Grahn & Stigsdotter (2010),
  N19 Hicks et al. (2020), N22 Joye & van den Berg (2011)
- 오픈 액세스 출판본(CC BY 4.0) 1편: N25 Chiorri et al. (2026)

엑셀·README 반영:
- 마스터 해당 행 확인 상태 → 원문 PDF 확인
- E20 저자 기입(Scott, Duncan & McCoy)
- 요약·자극 조건을 원문 기준으로 보강·정정
  (E20 표본·결과, N11 연구 1은 환경 상상·연구 2는 영상, N13·N19·N22 결과)
- 미확보 목록에서 6편 행 삭제 → 6편
- README 수치 갱신(82편 = 확보 76편 + 미확보 6편)

Refs #15

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
+++ b/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
@@ -1423,7 +1423,7 @@
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 / 저널·PubMed 본문</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 / 저널·PubMed 본문</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 / 저널 초록</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3274,7 @@
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>기전/Factor: PFA; evolutionary assumption critique; 관찰 결과: 이론적 가정</t>
+          <t>기전/Factor: PFA; evolutionary assumption critique; 관찰 결과: 회복 반응을 진화적 적응으로 보는 SRT 가정에 실증·개념적 근거가 약하다고 보고 처리 유창성 모델 제안</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>기전/Factor: PSD; serene; refuge; prospect; 관찰 결과: 선호; 스트레스 관련 지각</t>
+          <t>기전/Factor: PSD; serene; refuge; prospect; 관찰 결과: 일반 선호는 Serene이 가장 높고, 스트레스와는 Refuge·Nature 선호가 가장 강하게 연관</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>기전/Factor: fascination; being away; extent; compatibility; 관찰 결과: Restorative component ratings</t>
+          <t>기전/Factor: fascination; being away; extent; compatibility; 관찰 결과: being away가 물리적·심리적 이탈 2요인으로 나뉜 5요인 구조, 자연 환경이 모든 요인에서 도시보다 높음</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="K79" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 / 저널 초록</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Scott, Duncan &amp; McCoy</t>
         </is>
       </c>
       <c r="E95" s="5" t="n">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="H95" s="5" t="inlineStr">
         <is>
-          <t>자극/활동 Factor: Five Senses; 안내 방식; 매체: 오감 주의 관찰·교육; 결과: 시험 불안(TAQ)</t>
+          <t>자극/활동 Factor: Five Senses(5-4-3-2-1 그라운딩); 40분 교육 세션; 매체: 오감 주의 관찰·교육; 결과: 시험 불안(TAQ)</t>
         </is>
       </c>
       <c r="I95" s="5" t="inlineStr">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -6086,7 +6086,7 @@
       </c>
       <c r="K106" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -6291,7 +6291,7 @@
       </c>
       <c r="H110" s="5" t="inlineStr">
         <is>
-          <t>자극/활동 Factor: fascination; being away; extent; compatibility; 매체: 자연/도시 이미지·영상에 대한 구성요소 평정; 결과: Restorative component ratings</t>
+          <t>자극/활동 Factor: fascination; being away; extent; compatibility; 매체: 자연/도시 환경 상상(연구 1, 238명)·환경 영상(연구 2, 157명)에 대한 구성요소 평정; 결과: Restorative component ratings</t>
         </is>
       </c>
       <c r="I110" s="5" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="K110" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="K118" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -8263,7 +8263,7 @@
       </c>
       <c r="H146" s="5" t="inlineStr">
         <is>
-          <t>측정 지표: SART; Bayes factor; 결과요약: 자연 이미지의 주의력 회복 효과를 재현하지 못함</t>
+          <t>측정 지표: SART; Bayes factor; 결과요약: 자연 84명·도시 85명에서 자연 이미지의 주의력 회복 효과를 재현하지 못함(베이즈 분석도 영가설 지지)</t>
         </is>
       </c>
       <c r="I146" s="5" t="inlineStr">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="K146" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 / 저널 초록</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D151" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Scott, Duncan &amp; McCoy</t>
         </is>
       </c>
       <c r="E151" s="5" t="n">
@@ -8538,7 +8538,7 @@
       </c>
       <c r="H151" s="5" t="inlineStr">
         <is>
-          <t>측정 지표: 시험 불안(TAQ); 결과요약: 사전사후 시험불안 감소 보고</t>
+          <t>측정 지표: 시험 불안(TAQ); 결과요약: 간호학생 94명 참여·48명 사전사후 완료. TAQ 평균 4.7점 감소(p&lt;.001), 고불안 비율 23%→4%(p=.03)</t>
         </is>
       </c>
       <c r="I151" s="5" t="inlineStr">
@@ -8553,7 +8553,7 @@
       </c>
       <c r="K151" s="5" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="K178" s="6" t="inlineStr">
         <is>
-          <t>이번 회차 원문 미재검증</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -10588,7 +10588,7 @@
       </c>
       <c r="K188" s="6" t="inlineStr">
         <is>
-          <t>2026-10-22 / 저널·PubMed 본문</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
     </row>
@@ -11350,12 +11350,12 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>자연 이미지의 주의력 회복 효과를 재현하지 못함</t>
+          <t>자연/도시 이미지 25장(각 6초) 시청 전후 SART 비교에서 자연 이미지의 주의력 회복 효과를 재현하지 못함(자연 84명·도시 85명)</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 출판사/PubMed 근거 재확인(상세 수치 추가 정독)</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -11890,12 +11890,12 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>자연 선호·회복 이론의 진화론적 가정 검토</t>
+          <t>SRT의 진화론적 가정을 비판적으로 검토하고, 자연 회복 반응을 처리 유창성으로 설명하는 대안 모델 제시</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>미확인/원문 정독 필요</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -11950,12 +11950,12 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>지각된 자연 환경 특성의 주요 차원 도출</t>
+          <t>953명 우편 설문으로 8개 지각 차원 도출. Serene 선호가 가장 높고, 스트레스군에는 Refuge·Nature·Rich in Species 조합이 회복적일 수 있음</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>초록 확인</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -14323,7 +14323,7 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Scott, Duncan &amp; McCoy</t>
         </is>
       </c>
       <c r="E56" s="5" t="n">
@@ -14346,12 +14346,12 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>사전사후 시험불안 감소 보고</t>
+          <t>간호학생 대상 40분 교육(5-4-3-2-1 오감 그라운딩) 뒤 시험 전후 TAQ 4.7점 감소(p&lt;.001). 대조군 없는 단일군 설계</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>기존 조사; 원문 재검토</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
       <c r="K56" s="5" t="inlineStr">
@@ -15542,12 +15542,12 @@
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>지각된 자연 환경 특성의 주요 차원 도출</t>
+          <t>953명 우편 설문으로 8개 지각 차원 도출. Serene 선호가 가장 높고, 스트레스군에는 Refuge·Nature·Rich in Species 조합이 회복적일 수 있음</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>미확인/원문 정독 필요</t>
+          <t>2026-10-23 / 원문 PDF 확인</t>
         </is>
       </c>
       <c r="K76" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: fill missing authors for E18, E21 and N24 in master list
마스터 목록에서 저자가 "저자 원문 확인", "저자 정보 원문 확인"으로 비어 있던
13칸을 원문 PDF와 Crossref 기준으로 기입합니다. 저자가 4명 이상이면
기존 관례대로 et al.로 적습니다.

- E18 (2021, JPMH): Keenan et al. — 원고본에 저자가 없어 Crossref 기준
- E21 (2026, Appl Psychol Health Well-Being): Chen et al.
- N24 (2024, Internet Interventions): Fan & Baharum

Refs #17

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
+++ b/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
@@ -2926,7 +2926,7 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Chen et al.</t>
         </is>
       </c>
       <c r="E49" s="5" t="n">
@@ -5503,7 +5503,7 @@
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Chen et al.</t>
         </is>
       </c>
       <c r="E96" s="5" t="n">
@@ -6438,7 +6438,7 @@
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Fan &amp; Baharum</t>
         </is>
       </c>
       <c r="E113" s="5" t="n">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Keenan et al.</t>
         </is>
       </c>
       <c r="E115" s="5" t="n">
@@ -8575,7 +8575,7 @@
       </c>
       <c r="D152" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Chen et al.</t>
         </is>
       </c>
       <c r="E152" s="5" t="n">
@@ -8740,7 +8740,7 @@
       </c>
       <c r="D155" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Fan &amp; Baharum</t>
         </is>
       </c>
       <c r="E155" s="5" t="n">
@@ -9125,7 +9125,7 @@
       </c>
       <c r="D162" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Keenan et al.</t>
         </is>
       </c>
       <c r="E162" s="5" t="n">
@@ -11627,7 +11627,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Fan &amp; Baharum</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
@@ -13007,7 +13007,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Fan &amp; Baharum</t>
         </is>
       </c>
       <c r="E34" s="5" t="n">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Chen et al.</t>
         </is>
       </c>
       <c r="E48" s="5" t="n">
@@ -14443,7 +14443,7 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Keenan et al.</t>
         </is>
       </c>
       <c r="E58" s="5" t="n">
@@ -15279,7 +15279,7 @@
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Fan &amp; Baharum</t>
         </is>
       </c>
       <c r="E72" s="5" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>저자 원문 확인</t>
+          <t>Keenan et al.</t>
         </is>
       </c>
       <c r="E74" s="5" t="n">

</xml_diff>

<commit_message>
docs: fill missing authors for P12, P13, P14 and P19 in master list
같은 정리 중 저자가 "저자 정보 원문 확인"으로 비어 있던 6칸을 더 찾아
원문 PDF 첫 쪽 기준으로 기입합니다.

- P12 (2025, Psychological Medicine): Stenzel et al.
- P13 (2025, BMC Psychology): Wei et al.
- P14 (2024, npj Mental Health Research): Macrynikola et al.
- P19 (2024, Psychol Res Behav Manag): Muhammad Khir et al.

Refs #17

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
+++ b/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
@@ -1068,7 +1068,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Stenzel et al.</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Wei et al.</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Macrynikola et al.</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
@@ -6768,7 +6768,7 @@
       </c>
       <c r="D119" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Muhammad Khir et al.</t>
         </is>
       </c>
       <c r="E119" s="5" t="n">
@@ -10170,7 +10170,7 @@
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Macrynikola et al.</t>
         </is>
       </c>
       <c r="E181" s="6" t="n">
@@ -14623,7 +14623,7 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>저자 정보 원문 확인</t>
+          <t>Muhammad Khir et al.</t>
         </is>
       </c>
       <c r="E61" s="5" t="n">

</xml_diff>

<commit_message>
docs: fill missing DOIs for P12 and P19 in master list
마스터 목록 P12·P19 행의 비어 있던 DOI 3칸을 원문 PDF 기준으로 기입합니다.
Crossref에서 제목·저널·제1저자가 일치하는 것을 확인했고, 루트 엑셀
36편 목록(P19·P22)의 DOI와도 같습니다.

- P12 Stenzel et al. (2025): 10.1017/S0033291725000017
- P19 Muhammad Khir et al. (2024): 10.2147/PRBM.S437277

남은 빈 DOI는 DOI가 없는 P08(2004 국내 학회지)과 P32(학위논문)뿐입니다.

Refs #17

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
+++ b/LUMI_R_C_Research_2026-10-22/LUMI_R_C_논문목록_2026-10-22.xlsx
@@ -1089,7 +1089,11 @@
           <t>RNT의 정의·평가 도구</t>
         </is>
       </c>
-      <c r="I15" s="5" t="n"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>10.1017/S0033291725000017</t>
+        </is>
+      </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12017360/</t>
@@ -6789,7 +6793,11 @@
           <t>세션 기간·중재 조건</t>
         </is>
       </c>
-      <c r="I119" s="5" t="n"/>
+      <c r="I119" s="5" t="inlineStr">
+        <is>
+          <t>10.2147/PRBM.S437277</t>
+        </is>
+      </c>
       <c r="J119" s="5" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10844009/</t>
@@ -14654,7 +14662,11 @@
           <t>미확인/원문 정독 필요</t>
         </is>
       </c>
-      <c r="K61" s="5" t="n"/>
+      <c r="K61" s="5" t="inlineStr">
+        <is>
+          <t>10.2147/PRBM.S437277</t>
+        </is>
+      </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10844009/</t>

</xml_diff>